<commit_message>
Ground beam blinding at a uniform 0.50 m width
Each tie-beam piece is measured along its own axis between the footing/raft
blinding; blinding = total length x 0.50 m. DXF strips are 0.50 m wide with
each piece's length written on it; per-piece table in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/beam_blinding.xlsx
+++ b/beam_blinding.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,9 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -445,51 +449,1108 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ground beam concrete footprint (m²)</t>
+          <t>Blinding width taken for every tie beam (m)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80.73999999999999</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ground beam blinding, 100 mm each side, outside footing/raft blinding (m²)</t>
+          <t>Total beam length between footing/raft blinding (m)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>117.24</v>
+        <v>216.86</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Blinding volume @ 100 mm (m³)</t>
+          <t>Ground beam blinding = length x width (m²)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11.72</v>
+        <v>108.43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Equivalent length @ 0.50 m blinding width (m)</t>
+          <t>Blinding volume @ 100 mm (m³)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>234.5</v>
+        <v>10.84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Check: concrete + 100 mm each side (m²)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>115.39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Check: beam blinding as drawn on the plan (m²)</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B7" t="n">
         <v>121.39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Length (m)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Blinding @ width (m²)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Centre X</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Centre Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-22.55</v>
+      </c>
+      <c r="E10" t="n">
+        <v>55.36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-16.35</v>
+      </c>
+      <c r="E11" t="n">
+        <v>52.35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="E12" t="n">
+        <v>52.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E13" t="n">
+        <v>52.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-12.65</v>
+      </c>
+      <c r="E14" t="n">
+        <v>49.73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>49.73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>49.73</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-22.05</v>
+      </c>
+      <c r="E17" t="n">
+        <v>49.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-16.35</v>
+      </c>
+      <c r="E18" t="n">
+        <v>46.88</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="E19" t="n">
+        <v>47.13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E20" t="n">
+        <v>47.13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-38.79</v>
+      </c>
+      <c r="E21" t="n">
+        <v>45.21</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-28.95</v>
+      </c>
+      <c r="E22" t="n">
+        <v>44.68</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-12.95</v>
+      </c>
+      <c r="E23" t="n">
+        <v>43.99</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>43.99</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="E25" t="n">
+        <v>43.99</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D26" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="E26" t="n">
+        <v>43.99</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="D27" t="n">
+        <v>17.86</v>
+      </c>
+      <c r="E27" t="n">
+        <v>43.99</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-35.97</v>
+      </c>
+      <c r="E28" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="E29" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-12.95</v>
+      </c>
+      <c r="E30" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D32" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="E32" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>24</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D33" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="E33" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="D34" t="n">
+        <v>16.79</v>
+      </c>
+      <c r="E34" t="n">
+        <v>39.53</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-16.35</v>
+      </c>
+      <c r="E35" t="n">
+        <v>35.13</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="E36" t="n">
+        <v>35.38</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E37" t="n">
+        <v>35.25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C38" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-33.04</v>
+      </c>
+      <c r="E38" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-21.09</v>
+      </c>
+      <c r="E39" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>31</v>
+      </c>
+      <c r="B40" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-13.06</v>
+      </c>
+      <c r="E40" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>32</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-3.38</v>
+      </c>
+      <c r="E41" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>33</v>
+      </c>
+      <c r="B42" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E42" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>34</v>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="E43" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>35</v>
+      </c>
+      <c r="B44" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="D44" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="E44" t="n">
+        <v>30.53</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>36</v>
+      </c>
+      <c r="B45" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-16.35</v>
+      </c>
+      <c r="E45" t="n">
+        <v>26.01</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>37</v>
+      </c>
+      <c r="B46" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="E46" t="n">
+        <v>26.06</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>38</v>
+      </c>
+      <c r="B47" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E47" t="n">
+        <v>26.13</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>39</v>
+      </c>
+      <c r="B48" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-30.1</v>
+      </c>
+      <c r="E48" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>40</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-19.65</v>
+      </c>
+      <c r="E49" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-13.11</v>
+      </c>
+      <c r="E50" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>42</v>
+      </c>
+      <c r="B51" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="E51" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>43</v>
+      </c>
+      <c r="B52" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D52" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="E52" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>44</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="E53" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>45</v>
+      </c>
+      <c r="B54" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D54" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="E54" t="n">
+        <v>21.53</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>46</v>
+      </c>
+      <c r="B55" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D55" t="n">
+        <v>20.15</v>
+      </c>
+      <c r="E55" t="n">
+        <v>17.96</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-21.15</v>
+      </c>
+      <c r="E56" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-16.35</v>
+      </c>
+      <c r="E57" t="n">
+        <v>15.36</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>49</v>
+      </c>
+      <c r="B58" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="E58" t="n">
+        <v>14.96</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>50</v>
+      </c>
+      <c r="B59" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E59" t="n">
+        <v>14.98</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>51</v>
+      </c>
+      <c r="B60" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="D60" t="n">
+        <v>-33.94</v>
+      </c>
+      <c r="E60" t="n">
+        <v>14.21</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B61" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="D61" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="E61" t="n">
+        <v>9.390000000000001</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>53</v>
+      </c>
+      <c r="B62" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="D62" t="n">
+        <v>22.88</v>
+      </c>
+      <c r="E62" t="n">
+        <v>9.390000000000001</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>54</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="D63" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="E63" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>55</v>
+      </c>
+      <c r="B64" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="D64" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="E64" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>56</v>
+      </c>
+      <c r="B65" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D65" t="n">
+        <v>22.76</v>
+      </c>
+      <c r="E65" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>57</v>
+      </c>
+      <c r="B66" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="C66" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="D66" t="n">
+        <v>-8.449999999999999</v>
+      </c>
+      <c r="E66" t="n">
+        <v>4.86</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>58</v>
+      </c>
+      <c r="B67" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D67" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>59</v>
+      </c>
+      <c r="B68" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D68" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="E68" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>60</v>
+      </c>
+      <c r="B69" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C69" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D69" t="n">
+        <v>19.59</v>
+      </c>
+      <c r="E69" t="n">
+        <v>2.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>